<commit_message>
Table with Department Information
</commit_message>
<xml_diff>
--- a/CSC 4500 GitHub/Employees.xlsx
+++ b/CSC 4500 GitHub/Employees.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\AU\CSC 4500 GitHub\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{68DE1A36-46DC-44ED-ACD7-77C5C23AD5C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE41941F-9F1C-4D9D-B07F-337C856FB274}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1020" yWindow="1260" windowWidth="21765" windowHeight="13560" xr2:uid="{620D3336-13B9-4639-8A03-C1386B546856}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{620D3336-13B9-4639-8A03-C1386B546856}"/>
   </bookViews>
   <sheets>
     <sheet name="Employees" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="36">
   <si>
     <t>Name</t>
   </si>
@@ -116,6 +116,18 @@
   </si>
   <si>
     <t>(815) 555-0110</t>
+  </si>
+  <si>
+    <t>Department</t>
+  </si>
+  <si>
+    <t>Human Resources</t>
+  </si>
+  <si>
+    <t>Information Technology</t>
+  </si>
+  <si>
+    <t>Sales</t>
   </si>
 </sst>
 </file>
@@ -976,15 +988,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0180AC25-0E1C-4BAD-B8BC-ABA58B0364BA}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" customWidth="1"/>
     <col min="2" max="2" width="41.7109375" customWidth="1"/>
     <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="25.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -994,8 +1007,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>32</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1005,8 +1021,11 @@
       <c r="C2" t="s">
         <v>5</v>
       </c>
+      <c r="D2" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -1016,8 +1035,11 @@
       <c r="C3" t="s">
         <v>8</v>
       </c>
+      <c r="D3" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1027,8 +1049,11 @@
       <c r="C4" t="s">
         <v>11</v>
       </c>
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1038,8 +1063,11 @@
       <c r="C5" t="s">
         <v>14</v>
       </c>
+      <c r="D5" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -1049,8 +1077,11 @@
       <c r="C6" t="s">
         <v>17</v>
       </c>
+      <c r="D6" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -1060,8 +1091,11 @@
       <c r="C7" t="s">
         <v>20</v>
       </c>
+      <c r="D7" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1071,8 +1105,11 @@
       <c r="C8" t="s">
         <v>22</v>
       </c>
+      <c r="D8" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1082,8 +1119,11 @@
       <c r="C9" t="s">
         <v>25</v>
       </c>
+      <c r="D9" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -1093,8 +1133,11 @@
       <c r="C10" t="s">
         <v>28</v>
       </c>
+      <c r="D10" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>29</v>
       </c>
@@ -1103,6 +1146,9 @@
       </c>
       <c r="C11" t="s">
         <v>31</v>
+      </c>
+      <c r="D11" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replaced with Department ID
</commit_message>
<xml_diff>
--- a/CSC 4500 GitHub/Employees.xlsx
+++ b/CSC 4500 GitHub/Employees.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\AU\CSC 4500 GitHub\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE41941F-9F1C-4D9D-B07F-337C856FB274}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA22D90E-611B-4E8F-8821-4FD2C292BC21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{620D3336-13B9-4639-8A03-C1386B546856}"/>
+    <workbookView xWindow="1020" yWindow="1260" windowWidth="14910" windowHeight="11730" xr2:uid="{620D3336-13B9-4639-8A03-C1386B546856}"/>
   </bookViews>
   <sheets>
     <sheet name="Employees" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
   <si>
     <t>Name</t>
   </si>
@@ -118,16 +118,7 @@
     <t>(815) 555-0110</t>
   </si>
   <si>
-    <t>Department</t>
-  </si>
-  <si>
-    <t>Human Resources</t>
-  </si>
-  <si>
-    <t>Information Technology</t>
-  </si>
-  <si>
-    <t>Sales</t>
+    <t>Department ID</t>
   </si>
 </sst>
 </file>
@@ -994,7 +985,7 @@
     <col min="1" max="1" width="18.85546875" customWidth="1"/>
     <col min="2" max="2" width="41.7109375" customWidth="1"/>
     <col min="3" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="25.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -1021,8 +1012,8 @@
       <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
-        <v>33</v>
+      <c r="D2">
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -1035,8 +1026,8 @@
       <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="D3" t="s">
-        <v>34</v>
+      <c r="D3">
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1049,8 +1040,8 @@
       <c r="C4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" t="s">
-        <v>33</v>
+      <c r="D4">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1063,8 +1054,8 @@
       <c r="C5" t="s">
         <v>14</v>
       </c>
-      <c r="D5" t="s">
-        <v>35</v>
+      <c r="D5">
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1077,8 +1068,8 @@
       <c r="C6" t="s">
         <v>17</v>
       </c>
-      <c r="D6" t="s">
-        <v>34</v>
+      <c r="D6">
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1091,8 +1082,8 @@
       <c r="C7" t="s">
         <v>20</v>
       </c>
-      <c r="D7" t="s">
-        <v>35</v>
+      <c r="D7">
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1105,8 +1096,8 @@
       <c r="C8" t="s">
         <v>22</v>
       </c>
-      <c r="D8" t="s">
-        <v>33</v>
+      <c r="D8">
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1119,8 +1110,8 @@
       <c r="C9" t="s">
         <v>25</v>
       </c>
-      <c r="D9" t="s">
-        <v>35</v>
+      <c r="D9">
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1133,8 +1124,8 @@
       <c r="C10" t="s">
         <v>28</v>
       </c>
-      <c r="D10" t="s">
-        <v>34</v>
+      <c r="D10">
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1147,8 +1138,8 @@
       <c r="C11" t="s">
         <v>31</v>
       </c>
-      <c r="D11" t="s">
-        <v>34</v>
+      <c r="D11">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>